<commit_message>
Hola gente del futuro, actualizado funciones conectadas
</commit_message>
<xml_diff>
--- a/APP/static/archivos/Plantila Referencia Estudiantes.xlsx
+++ b/APP/static/archivos/Plantila Referencia Estudiantes.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>USUARIO</t>
   </si>
@@ -22,16 +22,10 @@
     <t>EMAIL</t>
   </si>
   <si>
-    <t>TIPO_PERFIL</t>
-  </si>
-  <si>
     <t>NOMBRE</t>
   </si>
   <si>
     <t>APELLIDO</t>
-  </si>
-  <si>
-    <t>CENTRO_EDUCACIONAL</t>
   </si>
   <si>
     <t>CURSO</t>
@@ -172,17 +166,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I2" displayName="Tabla_1" name="Tabla_1" id="1">
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:G2" displayName="Tabla_1" name="Tabla_1" id="1">
+  <tableColumns count="7">
     <tableColumn name="USUARIO" id="1"/>
     <tableColumn name="CONTRASEÑA" id="2"/>
     <tableColumn name="EMAIL" id="3"/>
-    <tableColumn name="TIPO_PERFIL" id="4"/>
-    <tableColumn name="NOMBRE" id="5"/>
-    <tableColumn name="APELLIDO" id="6"/>
-    <tableColumn name="CENTRO_EDUCACIONAL" id="7"/>
-    <tableColumn name="CURSO" id="8"/>
-    <tableColumn name="FECHA_NACIMIENTO" id="9"/>
+    <tableColumn name="NOMBRE" id="4"/>
+    <tableColumn name="APELLIDO" id="5"/>
+    <tableColumn name="CURSO" id="6"/>
+    <tableColumn name="FECHA_NACIMIENTO" id="7"/>
   </tableColumns>
   <tableStyleInfo name="CARGA ESTUDIANTE-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
@@ -389,9 +381,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="6" width="25.13"/>
-    <col customWidth="1" min="7" max="7" width="27.13"/>
-    <col customWidth="1" min="8" max="9" width="25.13"/>
+    <col customWidth="1" min="1" max="7" width="25.13"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
@@ -416,28 +406,14 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
-      <c r="D2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="3"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="3"/>
     </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="G2">
-      <formula1>"Centro Educacional Cardenal José María Caro"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D2">
-      <formula1>"ESTUDIANTE"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="H2">
+    <dataValidation type="list" allowBlank="1" sqref="F2">
       <formula1>"1° Medio,2° Medio,3° Medio,4°Medio,Vespertino,Egresado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>